<commit_message>
Revert bless-snapshots gate; keep auto-regen + snapshot assertion
User intent: codegen continues to write ddi.xml/tsv.tsv per example,
test_snapshots.py asserts driver output matches them. Tautology for
single-driver case (snapshot generator == test driver) is the known
limitation. Cross-driver tests (qwacback when wired) consume same
snapshots → real signal. Committed snapshots also serve as inspectable
PR artifacts and visual documentation.
</commit_message>
<xml_diff>
--- a/examples/grid/xlsform.xlsx
+++ b/examples/grid/xlsform.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Vendor DDI 2.5 XSD + CDL schematron; add XSD validation tests
schemas/xsd/      — official DDI-Codebook 2.5 XSD set (copied from
                    survey2ddi/tests/schemas — superset of qwacback/xml).
                    Source: https://ddialliance.org/Specification/DDI-Codebook/2.5/
schemas/schematron/ddi_custom_rules.sch
                  — CDL convention rules (copied from qwacback/schematron).

test_ddi_validation.py:
- test_ddi_snapshot_xsd_valid: every blessed examples/<id>/ddi.xml must
  parse + validate against DDI 2.5 codebook.xsd via lxml. 9/9 pass.
- test_ddi_snapshot_schematron: SKIP for now — bundled schematron uses
  queryBinding='xpath2' + fn:current() which lxml.isoschematron (xpath1)
  and pyschematron's elementpath don't support. qwacback's Java
  schematron-worker enforces it in prod. TODO: wire saxon-based processor.

Next: downstream sync. qwacback and survey2ddi should pull schemas
from this repo at pinned tag instead of vendoring locally.
</commit_message>
<xml_diff>
--- a/examples/grid/xlsform.xlsx
+++ b/examples/grid/xlsform.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Auto-generate docs.md per v1-blessed type via codegen
For each QuestionType with tier='v1-blessed', codegen.py now emits
types/<slug>/docs.md containing:
- Tier + frozenSince
- Concept facets (openness/cardinality/dataNature)
- Cross-format mapping table (XLSForm / LS code / DDI intrvl / RD type /
  varFormat type / qwacback answerType)
- Lifecycle Mermaid diagram (XLSForm → LS TSV, XLSForm ↔ DDI)
- Variants table (linking to per-variant example dirs)
- Constraints (name length + pattern, choice code length, warnings)
- Round-trip safety table
- Test pointers
- Source pointers

Files marked GENERATED with note pointing to definition.jsonld as source.
5 docs written: integer, text, date, select_one, select_multiple.
</commit_message>
<xml_diff>
--- a/examples/grid/xlsform.xlsx
+++ b/examples/grid/xlsform.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="survey" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="choices" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="survey" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>